<commit_message>
Version 3.0, Modulos de Red Transaccional y Acciones de Mitigacion agregados
</commit_message>
<xml_diff>
--- a/Transacciones_AML_200.xlsx
+++ b/Transacciones_AML_200.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hobeddiaz/Documents/AML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5AA191-C7C8-2E41-AD25-D7D941CAF76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED043D12-7C21-194B-81A4-BA91E2F6F5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="20" windowWidth="23160" windowHeight="15260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="150">
   <si>
     <t>Cliente</t>
   </si>
@@ -483,6 +483,9 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Cliente_Destino</t>
   </si>
 </sst>
 </file>
@@ -525,7 +528,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -548,18 +551,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -865,7 +882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I201"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
@@ -873,9 +890,10 @@
     <col min="5" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -903,8 +921,11 @@
       <c r="I1" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>46037</v>
       </c>
@@ -932,8 +953,11 @@
       <c r="I2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>46063</v>
       </c>
@@ -961,8 +985,11 @@
       <c r="I3" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>46086</v>
       </c>
@@ -990,8 +1017,11 @@
       <c r="I4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>46042</v>
       </c>
@@ -1019,8 +1049,11 @@
       <c r="I5" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>46047</v>
       </c>
@@ -1048,8 +1081,11 @@
       <c r="I6" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>46067</v>
       </c>
@@ -1077,8 +1113,11 @@
       <c r="I7" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>46027</v>
       </c>
@@ -1106,8 +1145,11 @@
       <c r="I8" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>46071</v>
       </c>
@@ -1135,8 +1177,11 @@
       <c r="I9" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>46093</v>
       </c>
@@ -1164,8 +1209,11 @@
       <c r="I10" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>46096</v>
       </c>
@@ -1193,8 +1241,11 @@
       <c r="I11" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>46033</v>
       </c>
@@ -1222,8 +1273,11 @@
       <c r="I12" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>46073</v>
       </c>
@@ -1251,8 +1305,11 @@
       <c r="I13" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>46052</v>
       </c>
@@ -1280,8 +1337,11 @@
       <c r="I14" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>46058</v>
       </c>
@@ -1309,8 +1369,11 @@
       <c r="I15" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>46082</v>
       </c>
@@ -1338,8 +1401,11 @@
       <c r="I16" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>46091</v>
       </c>
@@ -1367,8 +1433,11 @@
       <c r="I17" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>46036</v>
       </c>
@@ -1396,8 +1465,11 @@
       <c r="I18" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>46075</v>
       </c>
@@ -1425,8 +1497,11 @@
       <c r="I19" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>46081</v>
       </c>
@@ -1454,8 +1529,11 @@
       <c r="I20" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J20" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>46086</v>
       </c>
@@ -1483,8 +1561,11 @@
       <c r="I21" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J21" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>46041</v>
       </c>
@@ -1512,8 +1593,11 @@
       <c r="I22" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46101</v>
       </c>
@@ -1541,8 +1625,11 @@
       <c r="I23" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>46030</v>
       </c>
@@ -1570,8 +1657,11 @@
       <c r="I24" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>46068</v>
       </c>
@@ -1599,8 +1689,11 @@
       <c r="I25" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>46083</v>
       </c>
@@ -1628,8 +1721,11 @@
       <c r="I26" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J26" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>46099</v>
       </c>
@@ -1657,8 +1753,11 @@
       <c r="I27" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>46044</v>
       </c>
@@ -1686,8 +1785,11 @@
       <c r="I28" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>46064</v>
       </c>
@@ -1715,8 +1817,11 @@
       <c r="I29" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>46054</v>
       </c>
@@ -1744,8 +1849,11 @@
       <c r="I30" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>46103</v>
       </c>
@@ -1773,8 +1881,11 @@
       <c r="I31" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>46032</v>
       </c>
@@ -1802,8 +1913,11 @@
       <c r="I32" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>46078</v>
       </c>
@@ -1831,8 +1945,11 @@
       <c r="I33" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J33" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>46063</v>
       </c>
@@ -1860,8 +1977,11 @@
       <c r="I34" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>46116</v>
       </c>
@@ -1889,8 +2009,11 @@
       <c r="I35" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J35" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>46089</v>
       </c>
@@ -1918,8 +2041,11 @@
       <c r="I36" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J36" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>46065</v>
       </c>
@@ -1947,8 +2073,11 @@
       <c r="I37" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J37" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>46094</v>
       </c>
@@ -1976,8 +2105,11 @@
       <c r="I38" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>46090</v>
       </c>
@@ -2005,8 +2137,11 @@
       <c r="I39" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J39" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>46030</v>
       </c>
@@ -2034,8 +2169,11 @@
       <c r="I40" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J40" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>46064</v>
       </c>
@@ -2063,8 +2201,11 @@
       <c r="I41" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>46140</v>
       </c>
@@ -2092,8 +2233,11 @@
       <c r="I42" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J42" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>46085</v>
       </c>
@@ -2121,8 +2265,11 @@
       <c r="I43" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J43" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>46024</v>
       </c>
@@ -2150,8 +2297,11 @@
       <c r="I44" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J44" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>46133</v>
       </c>
@@ -2179,8 +2329,11 @@
       <c r="I45" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J45" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>46074</v>
       </c>
@@ -2208,8 +2361,11 @@
       <c r="I46" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J46" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>46119</v>
       </c>
@@ -2237,8 +2393,11 @@
       <c r="I47" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J47" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>46081</v>
       </c>
@@ -2266,8 +2425,11 @@
       <c r="I48" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J48" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46135</v>
       </c>
@@ -2295,8 +2457,11 @@
       <c r="I49" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J49" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46139</v>
       </c>
@@ -2324,8 +2489,11 @@
       <c r="I50" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J50" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>46081</v>
       </c>
@@ -2353,8 +2521,11 @@
       <c r="I51" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J51" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>46126</v>
       </c>
@@ -2382,8 +2553,11 @@
       <c r="I52" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J52" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>46037</v>
       </c>
@@ -2411,8 +2585,11 @@
       <c r="I53" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J53" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>46036</v>
       </c>
@@ -2440,8 +2617,11 @@
       <c r="I54" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J54" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>46045</v>
       </c>
@@ -2469,8 +2649,11 @@
       <c r="I55" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J55" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>46076</v>
       </c>
@@ -2498,8 +2681,11 @@
       <c r="I56" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J56" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>46026</v>
       </c>
@@ -2527,8 +2713,11 @@
       <c r="I57" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J57" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>46101</v>
       </c>
@@ -2556,8 +2745,11 @@
       <c r="I58" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J58" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>46037</v>
       </c>
@@ -2585,8 +2777,11 @@
       <c r="I59" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J59" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>46141</v>
       </c>
@@ -2614,8 +2809,11 @@
       <c r="I60" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J60" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>46047</v>
       </c>
@@ -2643,8 +2841,11 @@
       <c r="I61" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J61" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>46064</v>
       </c>
@@ -2672,8 +2873,11 @@
       <c r="I62" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J62" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
         <v>46046</v>
       </c>
@@ -2701,8 +2905,11 @@
       <c r="I63" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J63" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
         <v>46034</v>
       </c>
@@ -2730,8 +2937,11 @@
       <c r="I64" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J64" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="2">
         <v>46070</v>
       </c>
@@ -2759,8 +2969,11 @@
       <c r="I65" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J65" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="2">
         <v>46078</v>
       </c>
@@ -2788,8 +3001,11 @@
       <c r="I66" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J66" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
         <v>46066</v>
       </c>
@@ -2817,8 +3033,11 @@
       <c r="I67" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J67" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="2">
         <v>46086</v>
       </c>
@@ -2846,8 +3065,11 @@
       <c r="I68" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J68" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>46098</v>
       </c>
@@ -2875,8 +3097,11 @@
       <c r="I69" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J69" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="2">
         <v>46097</v>
       </c>
@@ -2904,8 +3129,11 @@
       <c r="I70" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J70" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="2">
         <v>46065</v>
       </c>
@@ -2933,8 +3161,11 @@
       <c r="I71" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J71" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2">
         <v>46104</v>
       </c>
@@ -2962,8 +3193,11 @@
       <c r="I72" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J72" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2">
         <v>46052</v>
       </c>
@@ -2991,8 +3225,11 @@
       <c r="I73" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J73" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="2">
         <v>46030</v>
       </c>
@@ -3020,8 +3257,11 @@
       <c r="I74" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J74" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="2">
         <v>46118</v>
       </c>
@@ -3049,8 +3289,11 @@
       <c r="I75" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J75" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="2">
         <v>46099</v>
       </c>
@@ -3078,8 +3321,11 @@
       <c r="I76" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J76" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="2">
         <v>46083</v>
       </c>
@@ -3107,8 +3353,11 @@
       <c r="I77" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J77" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="2">
         <v>46078</v>
       </c>
@@ -3136,8 +3385,11 @@
       <c r="I78" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J78" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="2">
         <v>46117</v>
       </c>
@@ -3165,8 +3417,11 @@
       <c r="I79" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J79" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="2">
         <v>46119</v>
       </c>
@@ -3194,8 +3449,11 @@
       <c r="I80" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J80" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="2">
         <v>46127</v>
       </c>
@@ -3223,8 +3481,11 @@
       <c r="I81" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J81" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="2">
         <v>46065</v>
       </c>
@@ -3252,8 +3513,11 @@
       <c r="I82" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J82" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="2">
         <v>46141</v>
       </c>
@@ -3281,8 +3545,11 @@
       <c r="I83" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J83" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="2">
         <v>46090</v>
       </c>
@@ -3310,8 +3577,11 @@
       <c r="I84" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J84" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="2">
         <v>46080</v>
       </c>
@@ -3339,8 +3609,11 @@
       <c r="I85" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J85" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="2">
         <v>46092</v>
       </c>
@@ -3368,8 +3641,11 @@
       <c r="I86" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J86" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="2">
         <v>46103</v>
       </c>
@@ -3397,8 +3673,11 @@
       <c r="I87" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J87" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="2">
         <v>46113</v>
       </c>
@@ -3426,8 +3705,11 @@
       <c r="I88" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J88" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="2">
         <v>46070</v>
       </c>
@@ -3455,8 +3737,11 @@
       <c r="I89" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J89" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="2">
         <v>46139</v>
       </c>
@@ -3484,8 +3769,11 @@
       <c r="I90" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J90" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="2">
         <v>46122</v>
       </c>
@@ -3513,8 +3801,11 @@
       <c r="I91" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J91" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="2">
         <v>46099</v>
       </c>
@@ -3542,8 +3833,11 @@
       <c r="I92" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J92" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="2">
         <v>46068</v>
       </c>
@@ -3571,8 +3865,11 @@
       <c r="I93" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J93" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="2">
         <v>46139</v>
       </c>
@@ -3600,8 +3897,11 @@
       <c r="I94" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J94" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="2">
         <v>46130</v>
       </c>
@@ -3629,8 +3929,11 @@
       <c r="I95" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J95" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="2">
         <v>46123</v>
       </c>
@@ -3658,8 +3961,11 @@
       <c r="I96" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J96" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="2">
         <v>46099</v>
       </c>
@@ -3687,8 +3993,11 @@
       <c r="I97" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J97" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="2">
         <v>46053</v>
       </c>
@@ -3716,8 +4025,11 @@
       <c r="I98" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J98" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="2">
         <v>46088</v>
       </c>
@@ -3745,8 +4057,11 @@
       <c r="I99" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J99" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="2">
         <v>46026</v>
       </c>
@@ -3774,8 +4089,11 @@
       <c r="I100" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J100" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" s="2">
         <v>46045</v>
       </c>
@@ -3803,8 +4121,11 @@
       <c r="I101" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J101" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" s="2">
         <v>46086</v>
       </c>
@@ -3832,8 +4153,11 @@
       <c r="I102" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J102" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" s="2">
         <v>46100</v>
       </c>
@@ -3861,8 +4185,11 @@
       <c r="I103" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J103" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104" s="2">
         <v>46094</v>
       </c>
@@ -3890,8 +4217,11 @@
       <c r="I104" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J104" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" s="2">
         <v>46035</v>
       </c>
@@ -3919,8 +4249,11 @@
       <c r="I105" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J105" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" s="2">
         <v>46045</v>
       </c>
@@ -3948,8 +4281,11 @@
       <c r="I106" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J106" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107" s="2">
         <v>46074</v>
       </c>
@@ -3977,8 +4313,11 @@
       <c r="I107" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J107" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108" s="2">
         <v>46126</v>
       </c>
@@ -4006,8 +4345,11 @@
       <c r="I108" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J108" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109" s="2">
         <v>46087</v>
       </c>
@@ -4035,8 +4377,11 @@
       <c r="I109" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J109" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110" s="2">
         <v>46044</v>
       </c>
@@ -4064,8 +4409,11 @@
       <c r="I110" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J110" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111" s="2">
         <v>46084</v>
       </c>
@@ -4093,8 +4441,11 @@
       <c r="I111" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J111" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112" s="2">
         <v>46079</v>
       </c>
@@ -4122,8 +4473,11 @@
       <c r="I112" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J112" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A113" s="2">
         <v>46101</v>
       </c>
@@ -4151,8 +4505,11 @@
       <c r="I113" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J113" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A114" s="2">
         <v>46066</v>
       </c>
@@ -4180,8 +4537,11 @@
       <c r="I114" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J114" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A115" s="2">
         <v>46075</v>
       </c>
@@ -4209,8 +4569,11 @@
       <c r="I115" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J115" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A116" s="2">
         <v>46114</v>
       </c>
@@ -4238,8 +4601,11 @@
       <c r="I116" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J116" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A117" s="2">
         <v>46032</v>
       </c>
@@ -4267,8 +4633,11 @@
       <c r="I117" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J117" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A118" s="2">
         <v>46025</v>
       </c>
@@ -4296,8 +4665,11 @@
       <c r="I118" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J118" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119" s="2">
         <v>46103</v>
       </c>
@@ -4325,8 +4697,11 @@
       <c r="I119" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J119" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A120" s="2">
         <v>46110</v>
       </c>
@@ -4354,8 +4729,11 @@
       <c r="I120" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J120" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A121" s="2">
         <v>46088</v>
       </c>
@@ -4383,8 +4761,11 @@
       <c r="I121" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J121" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A122" s="2">
         <v>46029</v>
       </c>
@@ -4412,8 +4793,11 @@
       <c r="I122" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J122" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A123" s="2">
         <v>46111</v>
       </c>
@@ -4441,8 +4825,11 @@
       <c r="I123" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J123" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A124" s="2">
         <v>46096</v>
       </c>
@@ -4470,8 +4857,11 @@
       <c r="I124" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J124" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A125" s="2">
         <v>46084</v>
       </c>
@@ -4499,8 +4889,11 @@
       <c r="I125" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J125" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A126" s="2">
         <v>46080</v>
       </c>
@@ -4528,8 +4921,11 @@
       <c r="I126" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J126" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A127" s="2">
         <v>46087</v>
       </c>
@@ -4557,8 +4953,11 @@
       <c r="I127" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J127" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A128" s="2">
         <v>46098</v>
       </c>
@@ -4586,8 +4985,11 @@
       <c r="I128" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J128" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129" s="2">
         <v>46031</v>
       </c>
@@ -4615,8 +5017,11 @@
       <c r="I129" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J129" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130" s="2">
         <v>46125</v>
       </c>
@@ -4644,8 +5049,11 @@
       <c r="I130" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J130" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131" s="2">
         <v>46024</v>
       </c>
@@ -4673,8 +5081,11 @@
       <c r="I131" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J131" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132" s="2">
         <v>46140</v>
       </c>
@@ -4702,8 +5113,11 @@
       <c r="I132" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J132" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133" s="2">
         <v>46042</v>
       </c>
@@ -4731,8 +5145,11 @@
       <c r="I133" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J133" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134" s="2">
         <v>46041</v>
       </c>
@@ -4760,8 +5177,11 @@
       <c r="I134" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J134" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135" s="2">
         <v>46132</v>
       </c>
@@ -4789,8 +5209,11 @@
       <c r="I135" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J135" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136" s="2">
         <v>46097</v>
       </c>
@@ -4818,8 +5241,11 @@
       <c r="I136" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J136" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137" s="2">
         <v>46127</v>
       </c>
@@ -4847,8 +5273,11 @@
       <c r="I137" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J137" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138" s="2">
         <v>46127</v>
       </c>
@@ -4876,8 +5305,11 @@
       <c r="I138" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J138" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139" s="2">
         <v>46047</v>
       </c>
@@ -4905,8 +5337,11 @@
       <c r="I139" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J139" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140" s="2">
         <v>46092</v>
       </c>
@@ -4934,8 +5369,11 @@
       <c r="I140" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J140" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141" s="2">
         <v>46127</v>
       </c>
@@ -4963,8 +5401,11 @@
       <c r="I141" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J141" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142" s="2">
         <v>46124</v>
       </c>
@@ -4992,8 +5433,11 @@
       <c r="I142" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J142" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143" s="2">
         <v>46045</v>
       </c>
@@ -5021,8 +5465,11 @@
       <c r="I143" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J143" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144" s="2">
         <v>46130</v>
       </c>
@@ -5050,8 +5497,11 @@
       <c r="I144" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J144" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145" s="2">
         <v>46078</v>
       </c>
@@ -5079,8 +5529,11 @@
       <c r="I145" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J145" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146" s="2">
         <v>46099</v>
       </c>
@@ -5108,8 +5561,11 @@
       <c r="I146" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J146" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147" s="2">
         <v>46034</v>
       </c>
@@ -5137,8 +5593,11 @@
       <c r="I147" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J147" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148" s="2">
         <v>46125</v>
       </c>
@@ -5166,8 +5625,11 @@
       <c r="I148" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J148" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149" s="2">
         <v>46079</v>
       </c>
@@ -5195,8 +5657,11 @@
       <c r="I149" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J149" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150" s="2">
         <v>46116</v>
       </c>
@@ -5224,8 +5689,11 @@
       <c r="I150" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J150" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151" s="2">
         <v>46070</v>
       </c>
@@ -5253,8 +5721,11 @@
       <c r="I151" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J151" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152" s="2">
         <v>46039</v>
       </c>
@@ -5282,8 +5753,11 @@
       <c r="I152" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J152" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153" s="2">
         <v>46030</v>
       </c>
@@ -5311,8 +5785,11 @@
       <c r="I153" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J153" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154" s="2">
         <v>46119</v>
       </c>
@@ -5340,8 +5817,11 @@
       <c r="I154" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J154" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155" s="2">
         <v>46053</v>
       </c>
@@ -5369,8 +5849,11 @@
       <c r="I155" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J155" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A156" s="2">
         <v>46035</v>
       </c>
@@ -5398,8 +5881,11 @@
       <c r="I156" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J156" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157" s="2">
         <v>46077</v>
       </c>
@@ -5427,8 +5913,11 @@
       <c r="I157" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J157" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158" s="2">
         <v>46093</v>
       </c>
@@ -5456,8 +5945,11 @@
       <c r="I158" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J158" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A159" s="2">
         <v>46053</v>
       </c>
@@ -5485,8 +5977,11 @@
       <c r="I159" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J159" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A160" s="2">
         <v>46091</v>
       </c>
@@ -5514,8 +6009,11 @@
       <c r="I160" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J160" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A161" s="2">
         <v>46132</v>
       </c>
@@ -5543,8 +6041,11 @@
       <c r="I161" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J161" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A162" s="2">
         <v>46122</v>
       </c>
@@ -5572,8 +6073,11 @@
       <c r="I162" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J162" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A163" s="2">
         <v>46090</v>
       </c>
@@ -5601,8 +6105,11 @@
       <c r="I163" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J163" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A164" s="2">
         <v>46119</v>
       </c>
@@ -5630,8 +6137,11 @@
       <c r="I164" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J164" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A165" s="2">
         <v>46133</v>
       </c>
@@ -5659,8 +6169,11 @@
       <c r="I165" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J165" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A166" s="2">
         <v>46084</v>
       </c>
@@ -5688,8 +6201,11 @@
       <c r="I166" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J166" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167" s="2">
         <v>46023</v>
       </c>
@@ -5717,8 +6233,11 @@
       <c r="I167" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J167" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A168" s="2">
         <v>46129</v>
       </c>
@@ -5746,8 +6265,11 @@
       <c r="I168" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J168" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A169" s="2">
         <v>46108</v>
       </c>
@@ -5775,8 +6297,11 @@
       <c r="I169" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J169" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A170" s="2">
         <v>46094</v>
       </c>
@@ -5804,8 +6329,11 @@
       <c r="I170" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J170" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A171" s="2">
         <v>46056</v>
       </c>
@@ -5833,8 +6361,11 @@
       <c r="I171" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J171" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A172" s="2">
         <v>46112</v>
       </c>
@@ -5862,8 +6393,11 @@
       <c r="I172" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J172" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A173" s="2">
         <v>46094</v>
       </c>
@@ -5891,8 +6425,11 @@
       <c r="I173" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J173" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174" s="2">
         <v>46138</v>
       </c>
@@ -5920,8 +6457,11 @@
       <c r="I174" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J174" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A175" s="2">
         <v>46072</v>
       </c>
@@ -5949,8 +6489,11 @@
       <c r="I175" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J175" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A176" s="2">
         <v>46035</v>
       </c>
@@ -5978,8 +6521,11 @@
       <c r="I176" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J176" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A177" s="2">
         <v>46104</v>
       </c>
@@ -6007,8 +6553,11 @@
       <c r="I177" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J177" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A178" s="2">
         <v>46037</v>
       </c>
@@ -6036,8 +6585,11 @@
       <c r="I178" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J178" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A179" s="2">
         <v>46132</v>
       </c>
@@ -6065,8 +6617,11 @@
       <c r="I179" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J179" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A180" s="2">
         <v>46059</v>
       </c>
@@ -6094,8 +6649,11 @@
       <c r="I180" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J180" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A181" s="2">
         <v>46136</v>
       </c>
@@ -6123,8 +6681,11 @@
       <c r="I181" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J181" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A182" s="2">
         <v>46073</v>
       </c>
@@ -6152,8 +6713,11 @@
       <c r="I182" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J182" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A183" s="2">
         <v>46095</v>
       </c>
@@ -6181,8 +6745,11 @@
       <c r="I183" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J183" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A184" s="2">
         <v>46037</v>
       </c>
@@ -6210,8 +6777,11 @@
       <c r="I184" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J184" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A185" s="2">
         <v>46065</v>
       </c>
@@ -6239,8 +6809,11 @@
       <c r="I185" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J185" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A186" s="2">
         <v>46135</v>
       </c>
@@ -6268,8 +6841,11 @@
       <c r="I186" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J186" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A187" s="2">
         <v>46049</v>
       </c>
@@ -6297,8 +6873,11 @@
       <c r="I187" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J187" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A188" s="2">
         <v>46026</v>
       </c>
@@ -6326,8 +6905,11 @@
       <c r="I188" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J188" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A189" s="2">
         <v>46030</v>
       </c>
@@ -6355,8 +6937,11 @@
       <c r="I189" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J189" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A190" s="2">
         <v>46072</v>
       </c>
@@ -6384,8 +6969,11 @@
       <c r="I190" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J190" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A191" s="2">
         <v>46109</v>
       </c>
@@ -6413,8 +7001,11 @@
       <c r="I191" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J191" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A192" s="2">
         <v>46113</v>
       </c>
@@ -6442,8 +7033,11 @@
       <c r="I192" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J192" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A193" s="2">
         <v>46072</v>
       </c>
@@ -6471,8 +7065,11 @@
       <c r="I193" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J193" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A194" s="2">
         <v>46050</v>
       </c>
@@ -6500,8 +7097,11 @@
       <c r="I194" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J194" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A195" s="2">
         <v>46036</v>
       </c>
@@ -6529,8 +7129,11 @@
       <c r="I195" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J195" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A196" s="2">
         <v>46027</v>
       </c>
@@ -6558,8 +7161,11 @@
       <c r="I196" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J196" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A197" s="2">
         <v>46061</v>
       </c>
@@ -6587,8 +7193,11 @@
       <c r="I197" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J197" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A198" s="2">
         <v>46027</v>
       </c>
@@ -6616,8 +7225,11 @@
       <c r="I198" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J198" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A199" s="2">
         <v>46089</v>
       </c>
@@ -6645,8 +7257,11 @@
       <c r="I199" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J199" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A200" s="2">
         <v>46076</v>
       </c>
@@ -6674,8 +7289,11 @@
       <c r="I200" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J200" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A201" s="2">
         <v>46129</v>
       </c>
@@ -6702,6 +7320,9 @@
       </c>
       <c r="I201" t="s">
         <v>142</v>
+      </c>
+      <c r="J201" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>